<commit_message>
Replace events-tracker.xlsx with the complete V4 workbook, structure lock removed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017vNZU4VCCwC4dAhWw7UnUh
</commit_message>
<xml_diff>
--- a/events-tracker.xlsx
+++ b/events-tracker.xlsx
@@ -5,11 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://classerasa-my.sharepoint.com/personal/m_serag_classera_com/Documents/AY26 Classera PS Training Unit Initiatives &amp; Activities/AY26-27 eLearning Plan/Outputs/plans-site V261001.7 Interactive Onboarding &amp; SFI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://classerasa-my.sharepoint.com/personal/m_serag_classera_com/Documents/AY26 Classera PS Training Unit Initiatives &amp; Activities/AY26-27 eLearning Plan/Outputs/plans-site V261005/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="11_B31D5C704978562888068C73A4A5265DB18A4F65" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC5E3910-BC54-4FFC-82C5-0A6DD4AD617B}"/>
-  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="GT6RTs28arVuVVbJHNVA+74tm3CsKtOX1/t6N1+DEjtxFsYZb8cyxWH4NbWlgRRSWqb+7Srluyl3yEyEHkL+fg==" workbookSaltValue="z6zQ5x9wttKwXo5UNctm4w==" workbookSpinCount="100000" lockStructure="1"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_B31D5C704978562888068C73A4A5265DB18A4F65" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A38B884-53AE-421E-91C6-7791C1EF11EB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2759,11 +2758,11 @@
       </c>
       <c r="D16" s="16">
         <f>COUNTIFS(Events!$U$2:$U$400,D$15)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="16">
         <f>COUNTIFS(Events!$U$2:$U$400,E$15)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F16" s="16">
         <f>COUNTIFS(Events!$U$2:$U$400,F$15)</f>
@@ -3458,7 +3457,7 @@
         <v>Published</v>
       </c>
       <c r="U5" s="30" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="V5" s="30" t="s">
         <v>466</v>
@@ -6407,7 +6406,7 @@
         <v>25</v>
       </c>
       <c r="V37" s="30" t="s">
-        <v>119</v>
+        <v>469</v>
       </c>
       <c r="W37" s="30"/>
       <c r="X37" s="31"/>

</xml_diff>